<commit_message>
update player number data in playernumber.xlsx
</commit_message>
<xml_diff>
--- a/playernumber.xlsx
+++ b/playernumber.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="29">
   <si>
     <t>活动编号</t>
   </si>
@@ -6335,8 +6335,8 @@
       <c r="D249" s="4">
         <v>98408</v>
       </c>
-      <c r="E249" s="5" t="s">
-        <v>10</v>
+      <c r="E249" s="5">
+        <v>6</v>
       </c>
       <c r="F249" s="5" t="s">
         <v>7</v>
@@ -6348,6 +6348,24 @@
     <row r="250" spans="1:7">
       <c r="A250" s="5">
         <v>323</v>
+      </c>
+      <c r="B250" s="2">
+        <v>46279</v>
+      </c>
+      <c r="C250" s="2">
+        <v>46285</v>
+      </c>
+      <c r="D250" s="4">
+        <v>42230</v>
+      </c>
+      <c r="E250" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F250" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G250" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="251" spans="1:7">
@@ -11474,8 +11492,25 @@
       <c r="A211" s="5">
         <v>323</v>
       </c>
-      <c r="F211" s="5"/>
-      <c r="G211" s="5"/>
+      <c r="B211" s="2">
+        <v>46279</v>
+      </c>
+      <c r="C211" s="2">
+        <v>46285</v>
+      </c>
+      <c r="D211" s="3">
+        <v>8356</v>
+      </c>
+      <c r="E211" s="7">
+        <f>D211/B服!D250</f>
+        <v>0.197868813639593</v>
+      </c>
+      <c r="F211" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G211" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="212" spans="1:7">
       <c r="A212" s="5">

</xml_diff>